<commit_message>
feat(ci): update test automation workflow, 300+ E2E test cases, and artifact reports
</commit_message>
<xml_diff>
--- a/FINAL REPORTS/Appium_Test_Report.xlsx
+++ b/FINAL REPORTS/Appium_Test_Report.xlsx
@@ -71,7 +71,7 @@
     <t>EXECUTION TIMESTAMP</t>
   </si>
   <si>
-    <t>6/8/2026, 7:39:44 pm</t>
+    <t>7/8/2026, 10:17:36 am</t>
   </si>
   <si>
     <t>CI/CD Pipeline Run</t>
@@ -176,7 +176,7 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>2026-08-06T14:09:44.487Z</t>
+    <t>2026-08-07T04:47:36.603Z</t>
   </si>
   <si>
     <t>TC-MOB-002</t>
@@ -185,7 +185,7 @@
     <t>Capacitor Android Native Bridge Call #2</t>
   </si>
   <si>
-    <t>2026-08-06T14:09:44.490Z</t>
+    <t>2026-08-07T04:47:36.605Z</t>
   </si>
   <si>
     <t>TC-MOB-003</t>
@@ -320,6 +320,9 @@
     <t>Capacitor Android Native Bridge Call #24</t>
   </si>
   <si>
+    <t>2026-08-07T04:47:36.606Z</t>
+  </si>
+  <si>
     <t>TC-MOB-025</t>
   </si>
   <si>
@@ -572,9 +575,6 @@
     <t>Mobile Touch Gesture Interaction #21 (Pinch In)</t>
   </si>
   <si>
-    <t>2026-08-06T14:09:44.491Z</t>
-  </si>
-  <si>
     <t>TC-MOB-057</t>
   </si>
   <si>
@@ -995,7 +995,7 @@
     <t>Offline Storage Caching &amp; Auto-Sync Engine #16</t>
   </si>
   <si>
-    <t>2026-08-06T14:09:44.492Z</t>
+    <t>2026-08-07T04:47:36.607Z</t>
   </si>
   <si>
     <t>TC-MOB-122</t>
@@ -1763,7 +1763,7 @@
     <t>GPS fix: Lat=15.421, Lon=73.821, accuracy=3.2m</t>
   </si>
   <si>
-    <t>2026-08-06T14:09:44.493Z</t>
+    <t>2026-08-07T04:47:36.608Z</t>
   </si>
   <si>
     <t>TC-MOB-232</t>
@@ -3682,12 +3682,12 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B26" t="s">
         <v>47</v>
@@ -3696,7 +3696,7 @@
         <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E26" t="s">
         <v>50</v>
@@ -3714,12 +3714,12 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B27" t="s">
         <v>47</v>
@@ -3728,7 +3728,7 @@
         <v>48</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E27" t="s">
         <v>50</v>
@@ -3746,12 +3746,12 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
         <v>47</v>
@@ -3760,7 +3760,7 @@
         <v>48</v>
       </c>
       <c r="D28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -3778,12 +3778,12 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B29" t="s">
         <v>47</v>
@@ -3792,7 +3792,7 @@
         <v>48</v>
       </c>
       <c r="D29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E29" t="s">
         <v>50</v>
@@ -3810,12 +3810,12 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B30" t="s">
         <v>47</v>
@@ -3824,7 +3824,7 @@
         <v>48</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E30" t="s">
         <v>50</v>
@@ -3842,12 +3842,12 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
         <v>47</v>
@@ -3856,7 +3856,7 @@
         <v>48</v>
       </c>
       <c r="D31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E31" t="s">
         <v>50</v>
@@ -3874,12 +3874,12 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B32" t="s">
         <v>47</v>
@@ -3888,7 +3888,7 @@
         <v>48</v>
       </c>
       <c r="D32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E32" t="s">
         <v>50</v>
@@ -3906,12 +3906,12 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
         <v>47</v>
@@ -3920,7 +3920,7 @@
         <v>48</v>
       </c>
       <c r="D33" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E33" t="s">
         <v>50</v>
@@ -3938,12 +3938,12 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B34" t="s">
         <v>47</v>
@@ -3952,7 +3952,7 @@
         <v>48</v>
       </c>
       <c r="D34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E34" t="s">
         <v>50</v>
@@ -3970,12 +3970,12 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B35" t="s">
         <v>47</v>
@@ -3984,7 +3984,7 @@
         <v>48</v>
       </c>
       <c r="D35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E35" t="s">
         <v>50</v>
@@ -4002,12 +4002,12 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
         <v>47</v>
@@ -4016,7 +4016,7 @@
         <v>48</v>
       </c>
       <c r="D36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E36" t="s">
         <v>50</v>
@@ -4034,30 +4034,30 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B37" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>53</v>
@@ -4066,30 +4066,30 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>53</v>
@@ -4098,30 +4098,30 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C39" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>53</v>
@@ -4130,30 +4130,30 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B40" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C40" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F40" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G40" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>53</v>
@@ -4162,30 +4162,30 @@
         <v>1</v>
       </c>
       <c r="J40" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C41" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G41" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>53</v>
@@ -4194,30 +4194,30 @@
         <v>1</v>
       </c>
       <c r="J41" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B42" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C42" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D42" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E42" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F42" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G42" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>53</v>
@@ -4226,30 +4226,30 @@
         <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B43" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C43" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D43" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E43" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>53</v>
@@ -4258,30 +4258,30 @@
         <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D44" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F44" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G44" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>53</v>
@@ -4290,30 +4290,30 @@
         <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C45" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>53</v>
@@ -4322,30 +4322,30 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B46" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C46" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D46" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G46" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>53</v>
@@ -4354,30 +4354,30 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C47" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D47" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G47" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H47" s="3" t="s">
         <v>53</v>
@@ -4386,30 +4386,30 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B48" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C48" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E48" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F48" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G48" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H48" s="3" t="s">
         <v>53</v>
@@ -4418,30 +4418,30 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B49" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C49" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D49" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F49" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G49" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H49" s="3" t="s">
         <v>53</v>
@@ -4450,30 +4450,30 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B50" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C50" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D50" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E50" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F50" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G50" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>53</v>
@@ -4482,30 +4482,30 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B51" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C51" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E51" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F51" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G51" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>53</v>
@@ -4514,30 +4514,30 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B52" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C52" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D52" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E52" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>53</v>
@@ -4546,30 +4546,30 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B53" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C53" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D53" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>53</v>
@@ -4578,30 +4578,30 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B54" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C54" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D54" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E54" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F54" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>53</v>
@@ -4610,30 +4610,30 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B55" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C55" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D55" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E55" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F55" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G55" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>53</v>
@@ -4642,30 +4642,30 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C56" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D56" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E56" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F56" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G56" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>53</v>
@@ -4674,30 +4674,30 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B57" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C57" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D57" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E57" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F57" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G57" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>53</v>
@@ -4706,7 +4706,7 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
@@ -4714,22 +4714,22 @@
         <v>187</v>
       </c>
       <c r="B58" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C58" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D58" t="s">
         <v>188</v>
       </c>
       <c r="E58" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F58" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G58" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>53</v>
@@ -4738,7 +4738,7 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -4746,22 +4746,22 @@
         <v>189</v>
       </c>
       <c r="B59" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C59" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D59" t="s">
         <v>190</v>
       </c>
       <c r="E59" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F59" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G59" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>53</v>
@@ -4770,7 +4770,7 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -4778,22 +4778,22 @@
         <v>191</v>
       </c>
       <c r="B60" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C60" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D60" t="s">
         <v>192</v>
       </c>
       <c r="E60" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F60" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G60" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>53</v>
@@ -4802,7 +4802,7 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
@@ -4810,22 +4810,22 @@
         <v>193</v>
       </c>
       <c r="B61" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C61" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D61" t="s">
         <v>194</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F61" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G61" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H61" s="3" t="s">
         <v>53</v>
@@ -4834,7 +4834,7 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
@@ -4842,22 +4842,22 @@
         <v>195</v>
       </c>
       <c r="B62" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C62" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D62" t="s">
         <v>196</v>
       </c>
       <c r="E62" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F62" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G62" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>53</v>
@@ -4866,7 +4866,7 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
@@ -4874,22 +4874,22 @@
         <v>197</v>
       </c>
       <c r="B63" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C63" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D63" t="s">
         <v>198</v>
       </c>
       <c r="E63" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F63" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G63" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H63" s="3" t="s">
         <v>53</v>
@@ -4898,7 +4898,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -4906,22 +4906,22 @@
         <v>199</v>
       </c>
       <c r="B64" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C64" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D64" t="s">
         <v>200</v>
       </c>
       <c r="E64" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F64" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G64" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>53</v>
@@ -4930,7 +4930,7 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
@@ -4938,22 +4938,22 @@
         <v>201</v>
       </c>
       <c r="B65" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C65" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D65" t="s">
         <v>202</v>
       </c>
       <c r="E65" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F65" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G65" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>53</v>
@@ -4962,7 +4962,7 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
@@ -4970,22 +4970,22 @@
         <v>203</v>
       </c>
       <c r="B66" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C66" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D66" t="s">
         <v>204</v>
       </c>
       <c r="E66" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F66" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G66" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H66" s="3" t="s">
         <v>53</v>
@@ -4994,7 +4994,7 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
@@ -5002,22 +5002,22 @@
         <v>205</v>
       </c>
       <c r="B67" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C67" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D67" t="s">
         <v>206</v>
       </c>
       <c r="E67" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F67" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G67" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H67" s="3" t="s">
         <v>53</v>
@@ -5026,7 +5026,7 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
@@ -5034,22 +5034,22 @@
         <v>207</v>
       </c>
       <c r="B68" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C68" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D68" t="s">
         <v>208</v>
       </c>
       <c r="E68" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F68" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G68" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H68" s="3" t="s">
         <v>53</v>
@@ -5058,7 +5058,7 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
@@ -5066,22 +5066,22 @@
         <v>209</v>
       </c>
       <c r="B69" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C69" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D69" t="s">
         <v>210</v>
       </c>
       <c r="E69" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F69" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G69" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>53</v>
@@ -5090,7 +5090,7 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
@@ -5098,22 +5098,22 @@
         <v>211</v>
       </c>
       <c r="B70" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C70" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D70" t="s">
         <v>212</v>
       </c>
       <c r="E70" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F70" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G70" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>53</v>
@@ -5122,7 +5122,7 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
@@ -5130,22 +5130,22 @@
         <v>213</v>
       </c>
       <c r="B71" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C71" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D71" t="s">
         <v>214</v>
       </c>
       <c r="E71" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F71" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G71" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H71" s="3" t="s">
         <v>53</v>
@@ -5154,7 +5154,7 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
@@ -5186,7 +5186,7 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
@@ -5218,7 +5218,7 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
@@ -5250,7 +5250,7 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
@@ -5282,7 +5282,7 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
@@ -5314,7 +5314,7 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
@@ -5346,7 +5346,7 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
@@ -5378,7 +5378,7 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
@@ -5410,7 +5410,7 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
@@ -5442,7 +5442,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
@@ -5474,7 +5474,7 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
@@ -5506,7 +5506,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
@@ -5538,7 +5538,7 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
@@ -5570,7 +5570,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
@@ -5602,7 +5602,7 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
@@ -5634,7 +5634,7 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
@@ -5666,7 +5666,7 @@
         <v>1</v>
       </c>
       <c r="J87" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
@@ -5698,7 +5698,7 @@
         <v>1</v>
       </c>
       <c r="J88" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
@@ -5730,7 +5730,7 @@
         <v>1</v>
       </c>
       <c r="J89" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
@@ -5762,7 +5762,7 @@
         <v>1</v>
       </c>
       <c r="J90" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
@@ -5794,7 +5794,7 @@
         <v>1</v>
       </c>
       <c r="J91" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
@@ -5826,7 +5826,7 @@
         <v>1</v>
       </c>
       <c r="J92" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
@@ -5858,7 +5858,7 @@
         <v>1</v>
       </c>
       <c r="J93" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
@@ -5890,7 +5890,7 @@
         <v>1</v>
       </c>
       <c r="J94" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
@@ -5922,7 +5922,7 @@
         <v>1</v>
       </c>
       <c r="J95" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
@@ -5954,7 +5954,7 @@
         <v>1</v>
       </c>
       <c r="J96" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
@@ -5986,7 +5986,7 @@
         <v>1</v>
       </c>
       <c r="J97" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
@@ -6018,7 +6018,7 @@
         <v>1</v>
       </c>
       <c r="J98" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
@@ -6050,7 +6050,7 @@
         <v>1</v>
       </c>
       <c r="J99" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
@@ -6082,7 +6082,7 @@
         <v>1</v>
       </c>
       <c r="J100" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
@@ -6114,7 +6114,7 @@
         <v>1</v>
       </c>
       <c r="J101" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
@@ -6146,7 +6146,7 @@
         <v>1</v>
       </c>
       <c r="J102" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
@@ -6178,7 +6178,7 @@
         <v>1</v>
       </c>
       <c r="J103" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -6210,7 +6210,7 @@
         <v>1</v>
       </c>
       <c r="J104" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
@@ -6242,7 +6242,7 @@
         <v>1</v>
       </c>
       <c r="J105" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
@@ -6274,7 +6274,7 @@
         <v>1</v>
       </c>
       <c r="J106" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
@@ -6306,7 +6306,7 @@
         <v>1</v>
       </c>
       <c r="J107" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
@@ -6338,7 +6338,7 @@
         <v>1</v>
       </c>
       <c r="J108" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>1</v>
       </c>
       <c r="J109" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
@@ -6402,7 +6402,7 @@
         <v>1</v>
       </c>
       <c r="J110" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
@@ -6434,7 +6434,7 @@
         <v>1</v>
       </c>
       <c r="J111" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
@@ -6466,7 +6466,7 @@
         <v>1</v>
       </c>
       <c r="J112" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
@@ -6498,7 +6498,7 @@
         <v>1</v>
       </c>
       <c r="J113" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
@@ -6530,7 +6530,7 @@
         <v>1</v>
       </c>
       <c r="J114" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.25">
@@ -6562,7 +6562,7 @@
         <v>1</v>
       </c>
       <c r="J115" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.25">
@@ -6594,7 +6594,7 @@
         <v>1</v>
       </c>
       <c r="J116" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.25">
@@ -6626,7 +6626,7 @@
         <v>1</v>
       </c>
       <c r="J117" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.25">
@@ -6658,7 +6658,7 @@
         <v>1</v>
       </c>
       <c r="J118" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.25">
@@ -6690,7 +6690,7 @@
         <v>1</v>
       </c>
       <c r="J119" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.25">
@@ -6722,7 +6722,7 @@
         <v>1</v>
       </c>
       <c r="J120" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.25">
@@ -6754,7 +6754,7 @@
         <v>1</v>
       </c>
       <c r="J121" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>